<commit_message>
Me cansa hacer esto
</commit_message>
<xml_diff>
--- a/ZAID_GASTOS.xlsx
+++ b/ZAID_GASTOS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NITRO\Desktop\MAC ZAID\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macair/Desktop/Windows_ZAID/DOC_Compartidos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2D593FF-19E8-4F42-A3E0-2D8C6F068FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A7C68A7-1BDD-E74A-B327-32DCAEADC34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="10320" xr2:uid="{0988253D-EE10-4ACA-AB6F-CAEBA60A6722}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{0988253D-EE10-4ACA-AB6F-CAEBA60A6722}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="50">
   <si>
     <t>SEMANA 3</t>
   </si>
@@ -184,6 +184,9 @@
   </si>
   <si>
     <t>Prueba de que se elimnie</t>
+  </si>
+  <si>
+    <t>ESTO ESTA ESCRITO EN LA MAC</t>
   </si>
 </sst>
 </file>
@@ -375,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -389,9 +392,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -410,29 +410,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -758,20 +748,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{290175BE-BD1E-4ABF-80F6-AA146AB0F03C}">
-  <dimension ref="A2:K47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:K49"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.21875" customWidth="1"/>
-    <col min="2" max="2" width="19.109375" customWidth="1"/>
-    <col min="3" max="3" width="19.77734375" customWidth="1"/>
-    <col min="4" max="4" width="18.5546875" customWidth="1"/>
+    <col min="1" max="1" width="14.1640625" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.5" customWidth="1"/>
     <col min="5" max="5" width="18.33203125" customWidth="1"/>
     <col min="6" max="6" width="17.33203125" customWidth="1"/>
-    <col min="7" max="7" width="15.21875" customWidth="1"/>
-    <col min="9" max="9" width="18.5546875" customWidth="1"/>
+    <col min="7" max="7" width="15.1640625" customWidth="1"/>
+    <col min="9" max="9" width="18.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -793,21 +783,21 @@
       <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="16" t="s">
+      <c r="J2" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="14" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>46118</v>
       </c>
-      <c r="B3" s="21">
+      <c r="B3" s="16">
         <v>200</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -816,44 +806,44 @@
       <c r="D3" s="4">
         <v>9.5</v>
       </c>
-      <c r="E3" s="21">
+      <c r="E3" s="16">
         <f>SUM(D3:D14)</f>
         <v>277.39999999999998</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="16">
         <f>B6-E3</f>
         <v>2.6000000000000227</v>
       </c>
-      <c r="G3" s="21">
+      <c r="G3" s="16">
         <f>F3</f>
         <v>2.6000000000000227</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="6">
+      <c r="J3" s="5">
         <v>7.5</v>
       </c>
-      <c r="K3" s="18">
+      <c r="K3" s="15">
         <f>SUM(J3:J12)</f>
         <v>72.900000000000006</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="22"/>
+      <c r="B4" s="17"/>
       <c r="C4" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="4">
         <v>8.5</v>
       </c>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="I4" s="9" t="s">
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="I4" s="8" t="s">
         <v>20</v>
       </c>
       <c r="J4" s="4">
@@ -861,18 +851,18 @@
       </c>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="10"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="7" t="s">
+    <row r="5" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="9"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="6" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="4">
         <v>13.5</v>
       </c>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
       <c r="I5" s="4" t="s">
         <v>21</v>
       </c>
@@ -881,24 +871,24 @@
       </c>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="12">
         <f>B3+B9+B10+B11</f>
         <v>280</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="4">
         <f>K3</f>
         <v>72.900000000000006</v>
       </c>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
       <c r="I6" s="4" t="s">
         <v>22</v>
       </c>
@@ -907,18 +897,18 @@
       </c>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
       <c r="C7" s="4" t="s">
         <v>28</v>
       </c>
       <c r="D7" s="4">
         <v>33</v>
       </c>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
       <c r="I7" s="4" t="s">
         <v>23</v>
       </c>
@@ -927,7 +917,7 @@
       </c>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4" t="s">
@@ -936,9 +926,9 @@
       <c r="D8" s="4">
         <v>60</v>
       </c>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
       <c r="I8" s="4" t="s">
         <v>25</v>
       </c>
@@ -947,7 +937,7 @@
       </c>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
@@ -971,7 +961,7 @@
       </c>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="4"/>
       <c r="B10" s="4">
         <v>30</v>
@@ -993,10 +983,10 @@
       </c>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="4">
@@ -1013,7 +1003,7 @@
       </c>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4" t="s">
@@ -1033,7 +1023,7 @@
       </c>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1042,10 +1032,7 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C14" s="12"/>
-    </row>
-    <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>29</v>
       </c>
@@ -1067,21 +1054,21 @@
       <c r="G21" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I21" s="15" t="s">
+      <c r="I21" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J21" s="15" t="s">
+      <c r="J21" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K21" s="16" t="s">
+      <c r="K21" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>46118</v>
       </c>
-      <c r="B22" s="21">
+      <c r="B22" s="16">
         <v>130</v>
       </c>
       <c r="C22" s="4" t="s">
@@ -1090,63 +1077,63 @@
       <c r="D22" s="4">
         <v>90</v>
       </c>
-      <c r="E22" s="21">
+      <c r="E22" s="16">
         <f>SUM(D22:D33)</f>
         <v>217.7</v>
       </c>
-      <c r="F22" s="21">
+      <c r="F22" s="16">
         <f>B25-E22</f>
         <v>12.300000000000011</v>
       </c>
-      <c r="G22" s="21">
+      <c r="G22" s="16">
         <f>F22+G3</f>
         <v>14.900000000000034</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="I22" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="J22" s="6">
+      <c r="J22" s="5">
         <v>2.2000000000000002</v>
       </c>
-      <c r="K22" s="18">
+      <c r="K22" s="15">
         <f>SUM(J22:J31)</f>
         <v>21.2</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="22"/>
+      <c r="B23" s="17"/>
       <c r="C23" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="4">
         <v>20</v>
       </c>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="I23" s="9" t="s">
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="I23" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="J23" s="9">
+      <c r="J23" s="8">
         <v>5</v>
       </c>
       <c r="K23" s="1"/>
     </row>
-    <row r="24" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="10"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="7" t="s">
+    <row r="24" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="9"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D24" s="4">
         <v>22</v>
       </c>
-      <c r="E24" s="23"/>
-      <c r="F24" s="23"/>
-      <c r="G24" s="23"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
       <c r="I24" s="4" t="s">
         <v>35</v>
       </c>
@@ -1155,23 +1142,23 @@
       </c>
       <c r="K24" s="1"/>
     </row>
-    <row r="25" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B25" s="14">
+      <c r="B25" s="12">
         <f>B22+B28+B29+B30+B31</f>
         <v>230</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D25" s="4">
         <v>10</v>
       </c>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
       <c r="I25" s="4" t="s">
         <v>37</v>
       </c>
@@ -1180,23 +1167,23 @@
       </c>
       <c r="K25" s="1"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" s="9"/>
-      <c r="B26" s="9"/>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
       <c r="C26" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D26" s="4">
         <v>15</v>
       </c>
-      <c r="E26" s="23"/>
-      <c r="F26" s="23"/>
-      <c r="G26" s="23"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
       <c r="K26" s="1"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4" t="s">
@@ -1205,21 +1192,21 @@
       <c r="D27" s="4">
         <v>10.5</v>
       </c>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
       <c r="K27" s="1"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="11">
+      <c r="B28" s="10">
         <v>100</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="10" t="s">
         <v>40</v>
       </c>
       <c r="D28" s="4">
@@ -1232,7 +1219,7 @@
       <c r="J28" s="4"/>
       <c r="K28" s="1"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4" t="s">
@@ -1248,10 +1235,10 @@
       <c r="J29" s="4"/>
       <c r="K29" s="1"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
-      <c r="C30" s="5"/>
+      <c r="C30" s="4"/>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
@@ -1260,7 +1247,7 @@
       <c r="J30" s="4"/>
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4" t="s">
@@ -1277,7 +1264,7 @@
       <c r="J31" s="4"/>
       <c r="K31" s="1"/>
     </row>
-    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>38</v>
       </c>
@@ -1299,21 +1286,21 @@
       <c r="G35" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I35" s="15" t="s">
+      <c r="I35" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J35" s="15" t="s">
+      <c r="J35" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K35" s="16" t="s">
+      <c r="K35" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>46118</v>
       </c>
-      <c r="B36" s="21">
+      <c r="B36" s="16">
         <v>85</v>
       </c>
       <c r="C36" s="4" t="s">
@@ -1322,103 +1309,103 @@
       <c r="D36" s="4">
         <v>32</v>
       </c>
-      <c r="E36" s="21">
+      <c r="E36" s="16">
         <f>SUM(D36:D47)</f>
         <v>204</v>
       </c>
-      <c r="F36" s="21">
+      <c r="F36" s="16">
         <f>B39-E36</f>
         <v>16</v>
       </c>
-      <c r="G36" s="21">
+      <c r="G36" s="16">
         <f>F36+G22</f>
         <v>30.900000000000034</v>
       </c>
-      <c r="I36" s="6" t="s">
+      <c r="I36" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="J36" s="6">
+      <c r="J36" s="5">
         <v>3</v>
       </c>
-      <c r="K36" s="18">
+      <c r="K36" s="15">
         <f>SUM(J36:J45)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B37" s="22"/>
+      <c r="B37" s="17"/>
       <c r="C37" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D37" s="4">
         <v>88</v>
       </c>
-      <c r="E37" s="23"/>
-      <c r="F37" s="23"/>
-      <c r="G37" s="23"/>
-      <c r="I37" s="20"/>
-      <c r="J37" s="20">
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8">
         <v>2</v>
       </c>
       <c r="K37" s="1"/>
     </row>
-    <row r="38" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="10"/>
-      <c r="B38" s="19"/>
-      <c r="C38" s="7" t="s">
+    <row r="38" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="9"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="6" t="s">
         <v>44</v>
       </c>
       <c r="D38" s="4">
         <v>22</v>
       </c>
-      <c r="E38" s="23"/>
-      <c r="F38" s="23"/>
-      <c r="G38" s="23"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
       <c r="K38" s="1"/>
     </row>
-    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="13" t="s">
+    <row r="39" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B39" s="14">
+      <c r="B39" s="12">
         <f>SUM(B42:B45,B36)</f>
         <v>220</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C39" s="6" t="s">
         <v>43</v>
       </c>
       <c r="D39" s="4">
         <v>15</v>
       </c>
-      <c r="E39" s="23"/>
-      <c r="F39" s="23"/>
-      <c r="G39" s="23"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="1"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A40" s="20"/>
-      <c r="B40" s="20"/>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40" s="8"/>
+      <c r="B40" s="8"/>
       <c r="C40" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D40" s="4">
         <v>12</v>
       </c>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="1"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4" t="s">
@@ -1427,21 +1414,21 @@
       <c r="D41" s="4">
         <v>12</v>
       </c>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="17"/>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="1"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B42" s="11">
+      <c r="B42" s="10">
         <v>100</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="10" t="s">
         <v>47</v>
       </c>
       <c r="D42" s="4">
@@ -1454,7 +1441,7 @@
       <c r="J42" s="4"/>
       <c r="K42" s="1"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" s="4"/>
       <c r="B43" s="4">
         <v>35</v>
@@ -1468,10 +1455,10 @@
       <c r="J43" s="4"/>
       <c r="K43" s="1"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
-      <c r="C44" s="5"/>
+      <c r="C44" s="4"/>
       <c r="D44" s="4"/>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
@@ -1480,7 +1467,7 @@
       <c r="J44" s="4"/>
       <c r="K44" s="1"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4" t="s">
@@ -1497,9 +1484,14 @@
       <c r="J45" s="4"/>
       <c r="K45" s="1"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ahora si, la real
</commit_message>
<xml_diff>
--- a/ZAID_GASTOS.xlsx
+++ b/ZAID_GASTOS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macair/Desktop/Windows_ZAID/DOC_Compartidos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NITRO\Desktop\MAC ZAID\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FEF66A5-6614-A541-898B-EA2CE1A5038F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{219A3BB7-5A11-415D-B5D6-434D4C4DBEBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{0988253D-EE10-4ACA-AB6F-CAEBA60A6722}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="10320" xr2:uid="{0988253D-EE10-4ACA-AB6F-CAEBA60A6722}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="54">
   <si>
     <t>SEMANA 3</t>
   </si>
@@ -196,6 +196,9 @@
   </si>
   <si>
     <t>Ahora si, el verdadero, habia olvidado hacer el push en el gitignore</t>
+  </si>
+  <si>
+    <t>Ahora me enviare esto a mi MAC</t>
   </si>
 </sst>
 </file>
@@ -757,20 +760,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{290175BE-BD1E-4ABF-80F6-AA146AB0F03C}">
-  <dimension ref="A2:K56"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A2:K58"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.1640625" customWidth="1"/>
-    <col min="2" max="2" width="19.1640625" customWidth="1"/>
-    <col min="3" max="3" width="19.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.5" customWidth="1"/>
+    <col min="1" max="1" width="14.109375" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" customWidth="1"/>
+    <col min="3" max="3" width="19.77734375" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" customWidth="1"/>
     <col min="5" max="5" width="18.33203125" customWidth="1"/>
     <col min="6" max="6" width="17.33203125" customWidth="1"/>
-    <col min="7" max="7" width="15.1640625" customWidth="1"/>
-    <col min="9" max="9" width="18.5" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
+    <col min="9" max="9" width="18.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -802,7 +805,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>46118</v>
       </c>
@@ -838,7 +841,7 @@
         <v>72.900000000000006</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>15</v>
       </c>
@@ -860,7 +863,7 @@
       </c>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
       <c r="B5" s="7"/>
       <c r="C5" s="6" t="s">
@@ -880,7 +883,7 @@
       </c>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>16</v>
       </c>
@@ -906,7 +909,7 @@
       </c>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="4" t="s">
@@ -926,7 +929,7 @@
       </c>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4" t="s">
@@ -946,7 +949,7 @@
       </c>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
@@ -970,7 +973,7 @@
       </c>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="4">
         <v>30</v>
@@ -992,7 +995,7 @@
       </c>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4" t="s">
@@ -1012,7 +1015,7 @@
       </c>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4" t="s">
@@ -1032,7 +1035,7 @@
       </c>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1041,7 +1044,7 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
-    <row r="21" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>29</v>
       </c>
@@ -1073,7 +1076,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>46118</v>
       </c>
@@ -1109,7 +1112,7 @@
         <v>21.2</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>15</v>
       </c>
@@ -1131,7 +1134,7 @@
       </c>
       <c r="K23" s="1"/>
     </row>
-    <row r="24" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="9"/>
       <c r="B24" s="7"/>
       <c r="C24" s="6" t="s">
@@ -1151,7 +1154,7 @@
       </c>
       <c r="K24" s="1"/>
     </row>
-    <row r="25" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="11" t="s">
         <v>16</v>
       </c>
@@ -1176,7 +1179,7 @@
       </c>
       <c r="K25" s="1"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="4" t="s">
@@ -1192,7 +1195,7 @@
       <c r="J26" s="4"/>
       <c r="K26" s="1"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4" t="s">
@@ -1208,7 +1211,7 @@
       <c r="J27" s="4"/>
       <c r="K27" s="1"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>14</v>
       </c>
@@ -1228,7 +1231,7 @@
       <c r="J28" s="4"/>
       <c r="K28" s="1"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4" t="s">
@@ -1244,7 +1247,7 @@
       <c r="J29" s="4"/>
       <c r="K29" s="1"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -1256,7 +1259,7 @@
       <c r="J30" s="4"/>
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4" t="s">
@@ -1273,7 +1276,7 @@
       <c r="J31" s="4"/>
       <c r="K31" s="1"/>
     </row>
-    <row r="35" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>38</v>
       </c>
@@ -1305,7 +1308,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>46118</v>
       </c>
@@ -1341,7 +1344,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>15</v>
       </c>
@@ -1361,7 +1364,7 @@
       </c>
       <c r="K37" s="1"/>
     </row>
-    <row r="38" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="9"/>
       <c r="B38" s="7"/>
       <c r="C38" s="6" t="s">
@@ -1377,7 +1380,7 @@
       <c r="J38" s="4"/>
       <c r="K38" s="1"/>
     </row>
-    <row r="39" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="11" t="s">
         <v>16</v>
       </c>
@@ -1398,7 +1401,7 @@
       <c r="J39" s="4"/>
       <c r="K39" s="1"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="4" t="s">
@@ -1414,7 +1417,7 @@
       <c r="J40" s="4"/>
       <c r="K40" s="1"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4" t="s">
@@ -1430,7 +1433,7 @@
       <c r="J41" s="4"/>
       <c r="K41" s="1"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>14</v>
       </c>
@@ -1450,7 +1453,7 @@
       <c r="J42" s="4"/>
       <c r="K42" s="1"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="4"/>
       <c r="B43" s="4">
         <v>35</v>
@@ -1464,7 +1467,7 @@
       <c r="J43" s="4"/>
       <c r="K43" s="1"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -1476,7 +1479,7 @@
       <c r="J44" s="4"/>
       <c r="K44" s="1"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4" t="s">
@@ -1493,29 +1496,34 @@
       <c r="J45" s="4"/>
       <c r="K45" s="1"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>